<commit_message>
20.05. Pred UAT automatizaciju
</commit_message>
<xml_diff>
--- a/testdata/data.xlsx
+++ b/testdata/data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8400"/>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="125">
   <si>
     <t>username</t>
   </si>
@@ -149,6 +149,18 @@
     <t>account_details_owner2</t>
   </si>
   <si>
+    <t>cards_item_debit_card_name</t>
+  </si>
+  <si>
+    <t>cards_item_debit_card_number</t>
+  </si>
+  <si>
+    <t>cards_item_credit_card_name</t>
+  </si>
+  <si>
+    <t>cards_item_credit_card_number</t>
+  </si>
+  <si>
     <t>Osir ANOEV</t>
   </si>
   <si>
@@ -335,6 +347,9 @@
     <t>0049015018282</t>
   </si>
   <si>
+    <t>Stambeni kredit</t>
+  </si>
+  <si>
     <t>0049038646620</t>
   </si>
   <si>
@@ -344,6 +359,18 @@
     <t>DRRE ĆEVMI</t>
   </si>
   <si>
+    <t>Visa PayWave - ROZALIJA ČOLIĆ</t>
+  </si>
+  <si>
+    <t>4381********1044</t>
+  </si>
+  <si>
+    <t>Master standard - ZUZANA KARAN</t>
+  </si>
+  <si>
+    <t>5309********0724</t>
+  </si>
+  <si>
     <t>Jail ĆEVGIMILĆ</t>
   </si>
   <si>
@@ -351,6 +378,30 @@
   </si>
   <si>
     <t>0049005001233</t>
+  </si>
+  <si>
+    <t>Icer OVIVL</t>
+  </si>
+  <si>
+    <t>205-9001004175165-12</t>
+  </si>
+  <si>
+    <t>205900100417516512</t>
+  </si>
+  <si>
+    <t>OVIVL OSIR</t>
+  </si>
+  <si>
+    <t>Vklaragan OVIT</t>
+  </si>
+  <si>
+    <t>205-9001004906720-69</t>
+  </si>
+  <si>
+    <t>205900100490672069</t>
+  </si>
+  <si>
+    <t>STANIŠA NIKOLA</t>
   </si>
 </sst>
 </file>
@@ -1377,8 +1428,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AN6"/>
-  <sheetFormatPr defaultColWidth="8.87962962962963" defaultRowHeight="14.4" outlineLevelRow="5"/>
+  <dimension ref="A1:AR8"/>
+  <sheetFormatPr defaultColWidth="8.87962962962963" defaultRowHeight="14.4" outlineLevelRow="7"/>
   <cols>
     <col min="1" max="1" width="17.75" customWidth="1"/>
     <col min="2" max="2" width="35.5555555555556" customWidth="1"/>
@@ -1413,9 +1464,12 @@
     <col min="37" max="37" width="23.7777777777778" customWidth="1"/>
     <col min="38" max="38" width="31.5555555555556" customWidth="1"/>
     <col min="39" max="40" width="22.1111111111111" customWidth="1"/>
+    <col min="41" max="42" width="27.8888888888889" customWidth="1"/>
+    <col min="43" max="43" width="31.7777777777778" customWidth="1"/>
+    <col min="44" max="44" width="27.8888888888889" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="1" spans="1:40">
+    <row r="1" customFormat="1" spans="1:44">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1536,612 +1590,952 @@
       <c r="AN1" t="s">
         <v>39</v>
       </c>
+      <c r="AO1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>43</v>
+      </c>
     </row>
-    <row r="2" customFormat="1" spans="1:40">
+    <row r="2" customFormat="1" spans="1:44">
       <c r="A2" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="F2" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I2" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="R2" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="V2" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="W2" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="X2" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Y2" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AB2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AC2" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="AD2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="AE2" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AF2" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AG2" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH2" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="AI2" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK2" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>75</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>76</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>54</v>
+      </c>
+      <c r="AO2" t="s">
+        <v>54</v>
+      </c>
+      <c r="AP2" t="s">
+        <v>54</v>
+      </c>
+      <c r="AQ2" t="s">
+        <v>54</v>
+      </c>
+      <c r="AR2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" customFormat="1" spans="1:44">
+      <c r="A3" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="C3" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="D3" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="M3" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q3" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="R3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="S3" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="U3" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="V3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="W3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="X3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Y3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Z3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AA3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AE3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AF3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AG3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AH3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AI3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AK3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AM3" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="AN3" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="AO3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AP3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AQ3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AR3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" customFormat="1" spans="1:44">
+      <c r="A4" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="I2" s="11" t="s">
+      <c r="C4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="E4" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="R4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="S4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="T4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="U4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="V4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="W4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="X4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Y4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Z4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AA4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AE4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AF4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AG4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AH4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AI4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AK4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AM4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AN4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AO4" t="s">
+        <v>54</v>
+      </c>
+      <c r="AP4" t="s">
+        <v>54</v>
+      </c>
+      <c r="AQ4" t="s">
+        <v>54</v>
+      </c>
+      <c r="AR4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" customFormat="1" spans="1:44">
+      <c r="A5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="K2" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="L2" s="1" t="s">
+      <c r="C5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="M2" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="O2" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="R2" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="T2" s="1" t="s">
+      <c r="G5" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="I5" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="N5" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="U2" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="V2" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="W2" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="X2" s="6" t="s">
+      <c r="O5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q5" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="R5" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="S5" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="T5" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="Y2" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z2" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="AA2" s="1" t="s">
+      <c r="U5" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="V5" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="W5" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="AB2" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="AC2" s="11" t="s">
+      <c r="X5" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="Y5" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="AD2" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="AE2" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AF2" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AG2" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="AH2" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="AI2" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="AJ2" t="s">
+      <c r="Z5" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="AA5" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="AB5" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="AC5" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="AD5" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="AE5" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="AF5" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AK2" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="AL2" t="s">
+      <c r="AG5" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="AM2" t="s">
-        <v>72</v>
-      </c>
-      <c r="AN2" t="s">
-        <v>50</v>
+      <c r="AH5" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AI5" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="AJ5" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AK5" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="AL5" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AM5" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="AN5" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="AO5" t="s">
+        <v>110</v>
+      </c>
+      <c r="AP5" t="s">
+        <v>111</v>
+      </c>
+      <c r="AQ5" t="s">
+        <v>112</v>
+      </c>
+      <c r="AR5" t="s">
+        <v>113</v>
       </c>
     </row>
-    <row r="3" customFormat="1" spans="1:40">
-      <c r="A3" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="F3" s="5" t="s">
+    <row r="6" s="1" customFormat="1" spans="1:44">
+      <c r="A6" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="G3" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="H3" s="5" t="s">
+      <c r="C6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="R6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="S6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="T6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="V6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="W6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="X6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Y6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Z6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AA6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC6" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="AD6" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="AE6" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="AF6" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="AG6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AH6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AI6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AK6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AM6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AN6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AO6" t="s">
+        <v>54</v>
+      </c>
+      <c r="AP6" t="s">
+        <v>54</v>
+      </c>
+      <c r="AQ6" t="s">
+        <v>54</v>
+      </c>
+      <c r="AR6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:44">
+      <c r="A7" t="s">
+        <v>117</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="I3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="K3" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="M3" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q3" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="R3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="S3" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="T3" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="U3" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="V3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="W3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="X3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="Y3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="Z3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AA3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AB3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AC3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AD3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AE3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AF3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AG3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AH3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AI3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AJ3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AK3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AL3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AM3" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="AN3" s="1" t="s">
-        <v>83</v>
+      <c r="C7" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="R7" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="S7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="T7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="U7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="V7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="W7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="X7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Y7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Z7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AA7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AE7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AF7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AG7" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="AH7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AI7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AK7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AM7" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="AN7" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="AO7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AP7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AQ7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AR7" t="s">
+        <v>54</v>
       </c>
     </row>
-    <row r="4" customFormat="1" spans="1:40">
-      <c r="A4" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="P4" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q4" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="R4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="S4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="T4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="U4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="V4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="W4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="X4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="Y4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="Z4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AA4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AB4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AC4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AD4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AE4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AF4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AG4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AH4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AI4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AJ4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AK4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AL4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AM4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AN4" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="5" customFormat="1" spans="1:40">
-      <c r="A5" t="s">
-        <v>87</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="E5" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="F5" s="1" t="s">
+    <row r="8" spans="1:44">
+      <c r="A8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B8" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="G5" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="I5" s="11" t="s">
+      <c r="C8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="R8" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="S8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="T8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="U8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="V8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="W8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="X8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Y8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Z8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AA8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AE8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AF8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AG8" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="J5" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="N5" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="O5" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="P5" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q5" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="R5" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="S5" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="T5" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="U5" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="V5" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="W5" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="X5" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="Y5" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z5" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="AA5" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="AB5" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="AC5" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="AD5" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="AE5" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="AF5" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="AG5" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH5" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AI5" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="AJ5" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AK5" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL5" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AM5" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="AN5" s="1" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="6" s="1" customFormat="1" spans="1:40">
-      <c r="A6" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="N6" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="O6" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="P6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="R6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="S6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="T6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="V6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="W6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="X6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="Y6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="Z6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AA6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AB6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AC6" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="AD6" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="AE6" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="AF6" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="AG6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AH6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AI6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AJ6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AK6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AL6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AM6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AN6" s="1" t="s">
-        <v>50</v>
+      <c r="AH8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AI8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AK8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AM8" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="AN8" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="AO8" t="s">
+        <v>54</v>
+      </c>
+      <c r="AP8" t="s">
+        <v>54</v>
+      </c>
+      <c r="AQ8" t="s">
+        <v>54</v>
+      </c>
+      <c r="AR8" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -2151,6 +2545,8 @@
     <hyperlink ref="B4" r:id="rId1" display="https://uat.dbp.nlb.si/web-retail/login" tooltip="https://uat.dbp.nlb.si/web-retail/login"/>
     <hyperlink ref="B5" r:id="rId1" display="https://uat.dbp.nlb.si/web-retail/login" tooltip="https://uat.dbp.nlb.si/web-retail/login"/>
     <hyperlink ref="B6" r:id="rId1" display="https://uat.dbp.nlb.si/web-retail/login" tooltip="https://uat.dbp.nlb.si/web-retail/login"/>
+    <hyperlink ref="B7" r:id="rId1" display="https://uat.dbp.nlb.si/web-retail/login" tooltip="https://uat.dbp.nlb.si/web-retail/login"/>
+    <hyperlink ref="B8" r:id="rId1" display="https://uat.dbp.nlb.si/web-retail/login" tooltip="https://uat.dbp.nlb.si/web-retail/login"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
18.08.2026 - stabilizovan deo testova
</commit_message>
<xml_diff>
--- a/testdata/data.xlsx
+++ b/testdata/data.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000"/>
+    <workbookView windowWidth="28800" windowHeight="11580"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="116">
   <si>
     <t>username</t>
   </si>
@@ -359,6 +359,9 @@
     <t>205-9001001626239-86</t>
   </si>
   <si>
+    <t>205-9001007668260-25</t>
+  </si>
+  <si>
     <t>0049018568496</t>
   </si>
   <si>
@@ -366,6 +369,12 @@
   </si>
   <si>
     <t>0049005001233</t>
+  </si>
+  <si>
+    <t>JAIL ĆEVGIMILĆ</t>
+  </si>
+  <si>
+    <t>Drre ĆEVMI</t>
   </si>
 </sst>
 </file>
@@ -1398,45 +1407,45 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AR9"/>
-  <sheetFormatPr defaultColWidth="8.87962962962963" defaultRowHeight="14.4"/>
+  <dimension ref="A1:AR10"/>
+  <sheetFormatPr defaultColWidth="8.87619047619048" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="17.75" customWidth="1"/>
-    <col min="2" max="2" width="35.5555555555556" customWidth="1"/>
-    <col min="3" max="3" width="7.75" customWidth="1"/>
-    <col min="4" max="4" width="11.25" customWidth="1"/>
-    <col min="5" max="5" width="22.4444444444444" customWidth="1"/>
-    <col min="6" max="6" width="19.1111111111111" customWidth="1"/>
+    <col min="1" max="1" width="17.752380952381" customWidth="1"/>
+    <col min="2" max="2" width="35.552380952381" customWidth="1"/>
+    <col min="3" max="3" width="7.75238095238095" customWidth="1"/>
+    <col min="4" max="4" width="11.247619047619" customWidth="1"/>
+    <col min="5" max="5" width="22.447619047619" customWidth="1"/>
+    <col min="6" max="6" width="19.1142857142857" customWidth="1"/>
     <col min="7" max="7" width="21" customWidth="1"/>
-    <col min="8" max="8" width="19.1111111111111" customWidth="1"/>
+    <col min="8" max="8" width="19.1142857142857" customWidth="1"/>
     <col min="9" max="9" width="21" customWidth="1"/>
-    <col min="10" max="10" width="19.1111111111111" customWidth="1"/>
-    <col min="11" max="11" width="38.7777777777778" customWidth="1"/>
-    <col min="12" max="12" width="40.1111111111111" customWidth="1"/>
-    <col min="13" max="14" width="33.8888888888889" customWidth="1"/>
-    <col min="15" max="15" width="28.8888888888889" customWidth="1"/>
-    <col min="16" max="17" width="30.4259259259259" customWidth="1"/>
-    <col min="18" max="18" width="37.8888888888889" customWidth="1"/>
-    <col min="19" max="19" width="27.8888888888889" customWidth="1"/>
-    <col min="20" max="20" width="30.4259259259259" customWidth="1"/>
+    <col min="10" max="10" width="19.1142857142857" customWidth="1"/>
+    <col min="11" max="11" width="38.7809523809524" customWidth="1"/>
+    <col min="12" max="12" width="40.1142857142857" customWidth="1"/>
+    <col min="13" max="14" width="33.8857142857143" customWidth="1"/>
+    <col min="15" max="15" width="28.8857142857143" customWidth="1"/>
+    <col min="16" max="17" width="30.4285714285714" customWidth="1"/>
+    <col min="18" max="18" width="37.8857142857143" customWidth="1"/>
+    <col min="19" max="19" width="27.8857142857143" customWidth="1"/>
+    <col min="20" max="20" width="30.4285714285714" customWidth="1"/>
     <col min="21" max="21" width="29.6666666666667" customWidth="1"/>
-    <col min="22" max="22" width="22.8888888888889" customWidth="1"/>
+    <col min="22" max="22" width="22.8857142857143" customWidth="1"/>
     <col min="23" max="24" width="24.6666666666667" customWidth="1"/>
-    <col min="25" max="28" width="33.2222222222222" customWidth="1"/>
-    <col min="29" max="29" width="21.2222222222222" customWidth="1"/>
-    <col min="30" max="30" width="19.4444444444444" customWidth="1"/>
-    <col min="31" max="31" width="22.4444444444444" customWidth="1"/>
-    <col min="32" max="32" width="19.4444444444444" customWidth="1"/>
-    <col min="33" max="33" width="23.7777777777778" customWidth="1"/>
-    <col min="34" max="34" width="31.5555555555556" customWidth="1"/>
-    <col min="35" max="35" width="23.7777777777778" customWidth="1"/>
-    <col min="36" max="36" width="31.5555555555556" customWidth="1"/>
-    <col min="37" max="37" width="23.7777777777778" customWidth="1"/>
-    <col min="38" max="38" width="31.5555555555556" customWidth="1"/>
-    <col min="39" max="40" width="22.1111111111111" customWidth="1"/>
-    <col min="41" max="42" width="27.8888888888889" customWidth="1"/>
-    <col min="43" max="43" width="31.7777777777778" customWidth="1"/>
-    <col min="44" max="44" width="27.8888888888889" customWidth="1"/>
+    <col min="25" max="28" width="33.2190476190476" customWidth="1"/>
+    <col min="29" max="29" width="21.2190476190476" customWidth="1"/>
+    <col min="30" max="30" width="19.447619047619" customWidth="1"/>
+    <col min="31" max="31" width="22.447619047619" customWidth="1"/>
+    <col min="32" max="32" width="19.447619047619" customWidth="1"/>
+    <col min="33" max="33" width="23.7809523809524" customWidth="1"/>
+    <col min="34" max="34" width="31.552380952381" customWidth="1"/>
+    <col min="35" max="35" width="23.7809523809524" customWidth="1"/>
+    <col min="36" max="36" width="31.552380952381" customWidth="1"/>
+    <col min="37" max="37" width="23.7809523809524" customWidth="1"/>
+    <col min="38" max="38" width="31.552380952381" customWidth="1"/>
+    <col min="39" max="40" width="22.1142857142857" customWidth="1"/>
+    <col min="41" max="42" width="27.8857142857143" customWidth="1"/>
+    <col min="43" max="43" width="31.7809523809524" customWidth="1"/>
+    <col min="44" max="44" width="27.8857142857143" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" spans="1:44">
@@ -2558,10 +2567,10 @@
         <v>109</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>54</v>
+        <v>110</v>
       </c>
       <c r="R9" s="1" t="s">
         <v>54</v>
@@ -2594,13 +2603,13 @@
         <v>54</v>
       </c>
       <c r="AC9" s="12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AD9" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="AE9" s="12" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AF9" s="1" t="s">
         <v>69</v>
@@ -2624,7 +2633,7 @@
         <v>54</v>
       </c>
       <c r="AM9" s="1" t="s">
-        <v>54</v>
+        <v>114</v>
       </c>
       <c r="AN9" s="1" t="s">
         <v>54</v>
@@ -2639,6 +2648,116 @@
         <v>54</v>
       </c>
       <c r="AR9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:44">
+      <c r="A10" t="s">
+        <v>115</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" t="s">
+        <v>54</v>
+      </c>
+      <c r="F10" t="s">
+        <v>54</v>
+      </c>
+      <c r="G10" t="s">
+        <v>54</v>
+      </c>
+      <c r="H10" t="s">
+        <v>54</v>
+      </c>
+      <c r="I10" t="s">
+        <v>54</v>
+      </c>
+      <c r="J10" t="s">
+        <v>54</v>
+      </c>
+      <c r="K10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L10" t="s">
+        <v>54</v>
+      </c>
+      <c r="M10" t="s">
+        <v>54</v>
+      </c>
+      <c r="N10" t="s">
+        <v>54</v>
+      </c>
+      <c r="O10" t="s">
+        <v>54</v>
+      </c>
+      <c r="P10" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>54</v>
+      </c>
+      <c r="R10" t="s">
+        <v>54</v>
+      </c>
+      <c r="S10" t="s">
+        <v>54</v>
+      </c>
+      <c r="T10" t="s">
+        <v>54</v>
+      </c>
+      <c r="U10" t="s">
+        <v>54</v>
+      </c>
+      <c r="V10" t="s">
+        <v>54</v>
+      </c>
+      <c r="W10" t="s">
+        <v>54</v>
+      </c>
+      <c r="X10" t="s">
+        <v>54</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>54</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>54</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD10" t="s">
+        <v>54</v>
+      </c>
+      <c r="AE10" t="s">
+        <v>54</v>
+      </c>
+      <c r="AF10" t="s">
+        <v>54</v>
+      </c>
+      <c r="AG10" t="s">
+        <v>54</v>
+      </c>
+      <c r="AH10" t="s">
+        <v>54</v>
+      </c>
+      <c r="AI10" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ10" t="s">
         <v>54</v>
       </c>
     </row>
@@ -2652,6 +2771,7 @@
     <hyperlink ref="B8" r:id="rId1" display="https://uat.dbp.nlb.si/web-retail/login" tooltip="https://uat.dbp.nlb.si/web-retail/login"/>
     <hyperlink ref="B9" r:id="rId1" display="https://uat.dbp.nlb.si/web-retail/login" tooltip="https://uat.dbp.nlb.si/web-retail/login"/>
     <hyperlink ref="B5" r:id="rId1" display="https://uat.dbp.nlb.si/web-retail/login" tooltip="https://uat.dbp.nlb.si/web-retail/login"/>
+    <hyperlink ref="B10" r:id="rId1" display="https://uat.dbp.nlb.si/web-retail/login" tooltip="https://uat.dbp.nlb.si/web-retail/login"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>